<commit_message>
feat: implement izin workflow module with database schema, models, and administrative management for pejabat
</commit_message>
<xml_diff>
--- a/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
+++ b/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
@@ -20,7 +20,7 @@
     <t>LAPORAN PRESENSI UKM UKM TAEKWONDO</t>
   </si>
   <si>
-    <t>Politeknik Pembangunan Pertanian Malang - Tanggal Cetak: 05/08/2026</t>
+    <t>Politeknik Pembangunan Pertanian Malang - Tanggal Cetak: 07/08/2026</t>
   </si>
   <si>
     <t>No</t>
@@ -44,13 +44,13 @@
     <t>Status Kehadiran</t>
   </si>
   <si>
-    <t>Yesenia Reichert</t>
+    <t>Prof. Aida Schmidt PhD</t>
   </si>
   <si>
     <t>Ujian Kenaikan Sabuk</t>
   </si>
   <si>
-    <t>05/08/2026</t>
+    <t>07/08/2026</t>
   </si>
   <si>
     <t>-</t>
@@ -467,7 +467,7 @@
         <v>9</v>
       </c>
       <c r="C5">
-        <v>5831408109</v>
+        <v>9314251482</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
feat: implement student permit application workflow with service, controller, and seeding logic
</commit_message>
<xml_diff>
--- a/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
+++ b/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
@@ -44,7 +44,7 @@
     <t>Status Kehadiran</t>
   </si>
   <si>
-    <t>Prof. Aida Schmidt PhD</t>
+    <t>Ezequiel Nolan III</t>
   </si>
   <si>
     <t>Ujian Kenaikan Sabuk</t>
@@ -467,7 +467,7 @@
         <v>9</v>
       </c>
       <c r="C5">
-        <v>9314251482</v>
+        <v>2907034595</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
feat: implement comprehensive student leave management system with PDF generation, approval workflows, and verification features
</commit_message>
<xml_diff>
--- a/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
+++ b/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
@@ -44,7 +44,7 @@
     <t>Status Kehadiran</t>
   </si>
   <si>
-    <t>Ezequiel Nolan III</t>
+    <t>Ron Friesen I</t>
   </si>
   <si>
     <t>Ujian Kenaikan Sabuk</t>
@@ -467,7 +467,7 @@
         <v>9</v>
       </c>
       <c r="C5">
-        <v>2907034595</v>
+        <v>2458417556</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
feat: implement administrative management for student permits including index, show views, and export functionality (M6)
</commit_message>
<xml_diff>
--- a/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
+++ b/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
   <si>
     <t>LAPORAN PRESENSI UKM UKM TAEKWONDO</t>
   </si>
@@ -44,7 +44,10 @@
     <t>Status Kehadiran</t>
   </si>
   <si>
-    <t>Myrna Miller</t>
+    <t>Ms. Ebony Zboncak</t>
+  </si>
+  <si>
+    <t>0917229484</t>
   </si>
   <si>
     <t>Ujian Kenaikan Sabuk</t>
@@ -466,20 +469,20 @@
       <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C5">
-        <v>6550147813</v>
+      <c r="C5" t="s">
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: clean up unused relationship method, import, and letter generation logic
</commit_message>
<xml_diff>
--- a/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
+++ b/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
@@ -44,10 +44,10 @@
     <t>Status Kehadiran</t>
   </si>
   <si>
-    <t>Ms. Ebony Zboncak</t>
-  </si>
-  <si>
-    <t>0917229484</t>
+    <t>Dr. Susanna Stracke</t>
+  </si>
+  <si>
+    <t>0896907333</t>
   </si>
   <si>
     <t>Ujian Kenaikan Sabuk</t>

</xml_diff>

<commit_message>
feat: implement workflow and operator role improvements and update project documentation
</commit_message>
<xml_diff>
--- a/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
+++ b/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
   <si>
     <t>LAPORAN PRESENSI UKM UKM TAEKWONDO</t>
   </si>
@@ -44,10 +44,7 @@
     <t>Status Kehadiran</t>
   </si>
   <si>
-    <t>Dr. Susanna Stracke</t>
-  </si>
-  <si>
-    <t>0896907333</t>
+    <t>Miss Mellie Kassulke V</t>
   </si>
   <si>
     <t>Ujian Kenaikan Sabuk</t>
@@ -469,20 +466,20 @@
       <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5">
+        <v>5450279300</v>
+      </c>
+      <c r="D5" t="s">
         <v>10</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>11</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>12</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>13</v>
-      </c>
-      <c r="G5" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add Dosen PA support to student management and implement QR payload decryption trait for secure scanning
</commit_message>
<xml_diff>
--- a/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
+++ b/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
@@ -15,12 +15,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
   <si>
     <t>LAPORAN PRESENSI UKM UKM TAEKWONDO</t>
   </si>
   <si>
-    <t>Politeknik Pembangunan Pertanian Malang - Tanggal Cetak: 08/08/2026</t>
+    <t>Politeknik Pembangunan Pertanian Malang - Tanggal Cetak: 06/09/2026</t>
+  </si>
+  <si>
+    <t>Rentang Tanggal: - s/d -</t>
   </si>
   <si>
     <t>No</t>
@@ -44,13 +47,13 @@
     <t>Status Kehadiran</t>
   </si>
   <si>
-    <t>Miss Mellie Kassulke V</t>
+    <t>Abigail Schimmel</t>
   </si>
   <si>
     <t>Ujian Kenaikan Sabuk</t>
   </si>
   <si>
-    <t>08/08/2026</t>
+    <t>06/09/2026</t>
   </si>
   <si>
     <t>-</t>
@@ -411,7 +414,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -436,56 +439,68 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
+    <row r="3" spans="1:7">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" t="s">
-        <v>8</v>
-      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6">
         <v>1</v>
       </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5">
-        <v>5450279300</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="B6" t="s">
         <v>10</v>
       </c>
-      <c r="E5" t="s">
+      <c r="C6">
+        <v>2196059553</v>
+      </c>
+      <c r="D6" t="s">
         <v>11</v>
       </c>
-      <c r="F5" t="s">
+      <c r="E6" t="s">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
+      <c r="F6" t="s">
         <v>13</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: implement QR payload encryption, add scoped authorization for officials, and introduce new feature tests
</commit_message>
<xml_diff>
--- a/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
+++ b/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
@@ -20,7 +20,7 @@
     <t>LAPORAN PRESENSI UKM UKM TAEKWONDO</t>
   </si>
   <si>
-    <t>Politeknik Pembangunan Pertanian Malang - Tanggal Cetak: 06/09/2026</t>
+    <t>Politeknik Pembangunan Pertanian Malang - Tanggal Cetak: 07/09/2026</t>
   </si>
   <si>
     <t>Rentang Tanggal: - s/d -</t>
@@ -47,13 +47,13 @@
     <t>Status Kehadiran</t>
   </si>
   <si>
-    <t>Abigail Schimmel</t>
+    <t>Moses Schmitt</t>
   </si>
   <si>
     <t>Ujian Kenaikan Sabuk</t>
   </si>
   <si>
-    <t>06/09/2026</t>
+    <t>07/09/2026</t>
   </si>
   <si>
     <t>-</t>
@@ -481,7 +481,7 @@
         <v>10</v>
       </c>
       <c r="C6">
-        <v>2196059553</v>
+        <v>6406496607</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
refactor: clean up route imports and update PejabatSeeder role ID
</commit_message>
<xml_diff>
--- a/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
+++ b/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
@@ -20,7 +20,7 @@
     <t>LAPORAN PRESENSI UKM UKM TAEKWONDO</t>
   </si>
   <si>
-    <t>Politeknik Pembangunan Pertanian Malang - Tanggal Cetak: 07/09/2026</t>
+    <t>Politeknik Pembangunan Pertanian Malang - Tanggal Cetak: 13/09/2026</t>
   </si>
   <si>
     <t>Rentang Tanggal: - s/d -</t>
@@ -47,13 +47,13 @@
     <t>Status Kehadiran</t>
   </si>
   <si>
-    <t>Moses Schmitt</t>
+    <t>Bailey Denesik</t>
   </si>
   <si>
     <t>Ujian Kenaikan Sabuk</t>
   </si>
   <si>
-    <t>07/09/2026</t>
+    <t>13/09/2026</t>
   </si>
   <si>
     <t>-</t>
@@ -481,7 +481,7 @@
         <v>10</v>
       </c>
       <c r="C6">
-        <v>6406496607</v>
+        <v>6222102924</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>

</xml_diff>